<commit_message>
Claims grants without duplicates; go-live configuration workbook with the sales activity masters
</commit_message>
<xml_diff>
--- a/docs/package/05_Delivery/Upload_Templates/GoLive_Configuration_Workbook.xlsx
+++ b/docs/package/05_Delivery/Upload_Templates/GoLive_Configuration_Workbook.xlsx
@@ -3909,7 +3909,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -3947,6 +3947,26 @@
       <b/>
       <sz val="11"/>
       <color rgb="FF006100"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFFFFFFF"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="14"/>
+      <color rgb="FF0B2A4A"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color rgb="FF5F6B76"/>
       <name val="Calibri"/>
       <family val="2"/>
     </font>
@@ -4028,9 +4048,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -4056,6 +4076,8 @@
     <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>

</xml_diff>